<commit_message>
docs: update SCRUM Backlog Export spreadsheet with latest requirements
</commit_message>
<xml_diff>
--- a/docs/requirement/SCRUM_Backlog_Export.xlsx
+++ b/docs/requirement/SCRUM_Backlog_Export.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngantran\source\repos\ecomerce\docs\requirement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74DBB1A-627B-41AA-868C-3A046D87ECE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8CCF02-BBD1-4A6C-9AE1-B3BD770CC61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2603,7 +2603,7 @@
         <v>54</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>83</v>
@@ -2691,7 +2691,7 @@
         <v>54</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>23</v>

</xml_diff>